<commit_message>
Fichier excel modifié comme l'original.
</commit_message>
<xml_diff>
--- a/Documents/Rappels/Rappels_2402.xlsx
+++ b/Documents/Rappels/Rappels_2402.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dossier Dev\Informatique\Gestcom\Documents\Rappels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{342322A9-AE49-49A4-A9C3-A0339F27B8D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B35C4027-D65E-4E6E-9340-A17DF1630003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4830" yWindow="990" windowWidth="21600" windowHeight="11295" firstSheet="3" activeTab="5" xr2:uid="{1B2651C3-EE09-40CE-BAC6-B64761F211A4}"/>
+    <workbookView xWindow="5835" yWindow="4185" windowWidth="21600" windowHeight="11295" firstSheet="3" activeTab="5" xr2:uid="{BF4CC841-7691-4FA8-9A94-200C91840CCF}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
     <t xml:space="preserve">      TB/PB</t>
   </si>
   <si>
-    <t>Le 16 juillet 2024</t>
+    <t>Le 17 juillet 2024</t>
   </si>
   <si>
     <t>Monsieur le Président</t>
@@ -209,13 +209,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
-    <numFmt numFmtId="164" formatCode="#\ ##0.000&quot;€&quot;"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="#\ ##0.000"/>
     <numFmt numFmtId="165" formatCode="#\ ##0.00"/>
-    <numFmt numFmtId="166" formatCode="#\ ##0.00&quot;€&quot;"/>
-    <numFmt numFmtId="167" formatCode="\-#\ ##0.00&quot;€&quot;"/>
-    <numFmt numFmtId="168" formatCode="#\ ##0.000"/>
-    <numFmt numFmtId="169" formatCode="#\ ##0.00,"/>
+    <numFmt numFmtId="166" formatCode="#\ ##0.00\ &quot;€&quot;"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -268,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -294,25 +291,16 @@
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -648,7 +636,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4775F077-C5DA-4811-9F47-4605AA88DC51}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17C9EE86-AC3F-4259-9BBC-C284B160E68D}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -657,7 +645,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96038322-E7B5-4B9A-B18E-A8283B8D4DFA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48763A49-C885-424D-AB6A-3BA39E20716B}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -757,6 +745,7 @@
         <v>15</v>
       </c>
       <c r="E31" s="6">
+        <f>ROUND(+K25/E25,2)</f>
         <v>10370.24</v>
       </c>
       <c r="F31" s="1" t="s">
@@ -767,8 +756,8 @@
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K33" s="11">
-        <v>46120800</v>
+      <c r="K33" s="10">
+        <v>-46120.800000000003</v>
       </c>
     </row>
     <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -777,7 +766,8 @@
         <v>17</v>
       </c>
       <c r="K35" s="8">
-        <v>26346437.120000001</v>
+        <f>SUM(K25,K33)</f>
+        <v>26346.440000000002</v>
       </c>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.2">
@@ -790,8 +780,9 @@
       <c r="J36" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K36" s="12">
-        <v>1449054.04</v>
+      <c r="K36" s="10">
+        <f>+K35*I36/100</f>
+        <v>1449.0542</v>
       </c>
     </row>
     <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -799,9 +790,9 @@
       <c r="G38" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K38" s="10">
-        <f>ROUND(SUM(K35:K36), 2)</f>
-        <v>27795491.16</v>
+      <c r="K38" s="9">
+        <f>SUM(K35:K36)</f>
+        <v>27795.494200000001</v>
       </c>
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.2">
@@ -833,8 +824,9 @@
       <c r="B51" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="H51" s="9">
-        <v>27795491.16</v>
+      <c r="H51" s="8">
+        <f>+K38</f>
+        <v>27795.494200000001</v>
       </c>
     </row>
   </sheetData>
@@ -843,7 +835,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E01989D-470B-47DD-A8CA-68121C526CF2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7A9BCB2-EF6E-4516-901B-38D5E4035D51}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -943,6 +935,7 @@
         <v>15</v>
       </c>
       <c r="E31" s="6">
+        <f>ROUND(+K25/E25,2)</f>
         <v>8465.5400000000009</v>
       </c>
       <c r="F31" s="1" t="s">
@@ -953,8 +946,8 @@
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K33" s="11">
-        <v>88294800</v>
+      <c r="K33" s="10">
+        <v>-88294.8</v>
       </c>
     </row>
     <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -963,7 +956,8 @@
         <v>17</v>
       </c>
       <c r="K35" s="8">
-        <v>24957194.120000001</v>
+        <f>SUM(K25,K33)</f>
+        <v>24957.190000000002</v>
       </c>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.2">
@@ -976,8 +970,9 @@
       <c r="J36" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K36" s="12">
-        <v>1372645.68</v>
+      <c r="K36" s="10">
+        <f>+K35*I36/100</f>
+        <v>1372.6454500000002</v>
       </c>
     </row>
     <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -985,9 +980,9 @@
       <c r="G38" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K38" s="10">
-        <f>ROUND(SUM(K35:K36), 2)</f>
-        <v>26329839.800000001</v>
+      <c r="K38" s="9">
+        <f>SUM(K35:K36)</f>
+        <v>26329.835450000002</v>
       </c>
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.2">
@@ -1019,8 +1014,9 @@
       <c r="B51" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="H51" s="9">
-        <v>26329839.800000001</v>
+      <c r="H51" s="8">
+        <f>+K38</f>
+        <v>26329.835450000002</v>
       </c>
     </row>
   </sheetData>
@@ -1029,7 +1025,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11029416-6BED-46B4-A511-1BB7B0C65090}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3501B4B-35BD-4364-A9ED-3A7DF86088A0}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1129,6 +1125,7 @@
         <v>15</v>
       </c>
       <c r="E31" s="6">
+        <f>ROUND(+K25/E25,2)</f>
         <v>8949.7999999999993</v>
       </c>
       <c r="F31" s="1" t="s">
@@ -1139,8 +1136,8 @@
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K33" s="11">
-        <v>176173800</v>
+      <c r="K33" s="10">
+        <v>-176173.8</v>
       </c>
     </row>
     <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1149,7 +1146,8 @@
         <v>17</v>
       </c>
       <c r="K35" s="8">
-        <v>62723211.399999999</v>
+        <f>SUM(K25,K33)</f>
+        <v>62723.210000000021</v>
       </c>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.2">
@@ -1162,8 +1160,9 @@
       <c r="J36" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K36" s="12">
-        <v>3449776.63</v>
+      <c r="K36" s="10">
+        <f>+K35*I36/100</f>
+        <v>3449.7765500000014</v>
       </c>
     </row>
     <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1171,9 +1170,9 @@
       <c r="G38" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K38" s="10">
-        <f>ROUND(SUM(K35:K36), 2)</f>
-        <v>66172988.030000001</v>
+      <c r="K38" s="9">
+        <f>SUM(K35:K36)</f>
+        <v>66172.986550000016</v>
       </c>
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.2">
@@ -1205,8 +1204,9 @@
       <c r="B51" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H51" s="9">
-        <v>66172988.030000001</v>
+      <c r="H51" s="8">
+        <f>+K38</f>
+        <v>66172.986550000016</v>
       </c>
     </row>
   </sheetData>
@@ -1215,7 +1215,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{118E910F-B509-4788-AA81-C8240B2A28A8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0742F98C-BE43-4AE4-875B-76E1058B8CF2}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1313,13 +1313,13 @@
       <c r="B26" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="14">
+      <c r="C26" s="11">
         <v>74</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E26" s="15">
+      <c r="E26" s="12">
         <v>2.9870000000000001</v>
       </c>
       <c r="F26" s="3" t="s">
@@ -1328,8 +1328,8 @@
       <c r="G26" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H26" s="13">
-        <v>6995600</v>
+      <c r="H26" s="7">
+        <v>6995.6</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>13</v>
@@ -1337,8 +1337,9 @@
       <c r="J26" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K26" s="12">
-        <v>20895796.16</v>
+      <c r="K26" s="10">
+        <f>ROUND(+E26*H26, 2)</f>
+        <v>20895.86</v>
       </c>
     </row>
     <row r="27" spans="2:11" ht="15" x14ac:dyDescent="0.25">
@@ -1356,9 +1357,9 @@
       <c r="F27" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K27" s="10">
+      <c r="K27" s="9">
         <f>SUM(K25:K26)</f>
-        <v>21061623.84</v>
+        <v>186723.53999999998</v>
       </c>
     </row>
     <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1367,7 +1368,8 @@
         <v>15</v>
       </c>
       <c r="E31" s="6">
-        <v>910615.41</v>
+        <f>ROUND(K27/E27,2)</f>
+        <v>8073.14</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>13</v>
@@ -1377,7 +1379,7 @@
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K33" s="11">
+      <c r="K33" s="10">
         <v>0</v>
       </c>
     </row>
@@ -1387,7 +1389,8 @@
         <v>17</v>
       </c>
       <c r="K35" s="8">
-        <v>21061623.84</v>
+        <f>SUM(K27,K33)</f>
+        <v>186723.53999999998</v>
       </c>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.2">
@@ -1400,8 +1403,9 @@
       <c r="J36" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K36" s="12">
-        <v>1158389.31</v>
+      <c r="K36" s="10">
+        <f>+K35*I36/100</f>
+        <v>10269.794699999999</v>
       </c>
     </row>
     <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1409,9 +1413,9 @@
       <c r="G38" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K38" s="10">
-        <f>ROUND(SUM(K35:K36), 2)</f>
-        <v>22220013.149999999</v>
+      <c r="K38" s="9">
+        <f>SUM(K35:K36)</f>
+        <v>196993.33469999998</v>
       </c>
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.2">
@@ -1443,8 +1447,9 @@
       <c r="B51" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="H51" s="9">
-        <v>22220013.149999999</v>
+      <c r="H51" s="8">
+        <f>+K38</f>
+        <v>196993.33469999998</v>
       </c>
     </row>
   </sheetData>
@@ -1453,7 +1458,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09632643-B00B-47D2-B482-A3AA5D7B7C71}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C0C6CB2-E0EA-43A6-B9F9-077E52785AB7}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1551,13 +1556,13 @@
       <c r="B26" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="14">
+      <c r="C26" s="11">
         <v>5</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E26" s="15">
+      <c r="E26" s="12">
         <v>0.20799999999999999</v>
       </c>
       <c r="F26" s="3" t="s">
@@ -1566,8 +1571,8 @@
       <c r="G26" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H26" s="13">
-        <v>7065600</v>
+      <c r="H26" s="7">
+        <v>7065.6</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>13</v>
@@ -1575,8 +1580,9 @@
       <c r="J26" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K26" s="12">
-        <v>1472670.18</v>
+      <c r="K26" s="10">
+        <f>ROUND(+E26*H26, 2)</f>
+        <v>1469.64</v>
       </c>
     </row>
     <row r="27" spans="2:11" ht="15" x14ac:dyDescent="0.25">
@@ -1594,9 +1600,9 @@
       <c r="F27" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K27" s="10">
+      <c r="K27" s="9">
         <f>SUM(K25:K26)</f>
-        <v>1597900.14</v>
+        <v>126699.6</v>
       </c>
     </row>
     <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1605,7 +1611,8 @@
         <v>15</v>
       </c>
       <c r="E31" s="6">
-        <v>103881.17</v>
+        <f>ROUND(K27/E27,2)</f>
+        <v>8236.8700000000008</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>13</v>
@@ -1615,7 +1622,7 @@
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K33" s="11">
+      <c r="K33" s="10">
         <v>0</v>
       </c>
     </row>
@@ -1625,7 +1632,8 @@
         <v>17</v>
       </c>
       <c r="K35" s="8">
-        <v>1597900.14</v>
+        <f>SUM(K27,K33)</f>
+        <v>126699.6</v>
       </c>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.2">
@@ -1638,8 +1646,9 @@
       <c r="J36" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K36" s="12">
-        <v>87884.51</v>
+      <c r="K36" s="10">
+        <f>+K35*I36/100</f>
+        <v>6968.4780000000001</v>
       </c>
     </row>
     <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1647,9 +1656,9 @@
       <c r="G38" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K38" s="10">
-        <f>ROUND(SUM(K35:K36), 2)</f>
-        <v>1685784.65</v>
+      <c r="K38" s="9">
+        <f>SUM(K35:K36)</f>
+        <v>133668.07800000001</v>
       </c>
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.2">
@@ -1681,8 +1690,9 @@
       <c r="B51" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="H51" s="9">
-        <v>1685784.65</v>
+      <c r="H51" s="8">
+        <f>+K38</f>
+        <v>133668.07800000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rappels avec prime A
</commit_message>
<xml_diff>
--- a/Documents/Rappels/Rappels_2402.xlsx
+++ b/Documents/Rappels/Rappels_2402.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dossier Dev\Informatique\Gestcom\Documents\Rappels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B35C4027-D65E-4E6E-9340-A17DF1630003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5EA33D97-C42D-4365-9E95-488695ED1F3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5835" yWindow="4185" windowWidth="21600" windowHeight="11295" firstSheet="3" activeTab="5" xr2:uid="{BF4CC841-7691-4FA8-9A94-200C91840CCF}"/>
+    <workbookView xWindow="2325" yWindow="2235" windowWidth="21600" windowHeight="11295" firstSheet="3" activeTab="5" xr2:uid="{D8AA5B2E-01EC-4C7C-8379-53BCEF521989}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="56">
   <si>
     <t xml:space="preserve">M PONCET FREDERIC        </t>
   </si>
@@ -155,6 +155,12 @@
   </si>
   <si>
     <t>25560 BANNANS</t>
+  </si>
+  <si>
+    <t>Prime qualité:</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
   <si>
     <t xml:space="preserve">PS : Nous virons ce jour, sur votre compte N° 0 0  </t>
@@ -265,7 +271,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -296,6 +302,9 @@
     </xf>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -636,7 +645,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17C9EE86-AC3F-4259-9BBC-C284B160E68D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE24BD8-54CD-41F6-8DAB-4C8E81FDCD62}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -645,7 +654,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48763A49-C885-424D-AB6A-3BA39E20716B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C598DBA3-A243-4CD2-A8BF-CEB75FEC3D0E}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -835,7 +844,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7A9BCB2-EF6E-4516-901B-38D5E4035D51}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F71F4056-B0CA-47D0-9DBC-DDC50849DC3B}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1025,7 +1034,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3501B4B-35BD-4364-A9ED-3A7DF86088A0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{401BF789-4F56-4F39-A2AC-AAB156D504D5}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1119,17 +1128,45 @@
         <v>238897.01</v>
       </c>
     </row>
+    <row r="27" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B27" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E27" s="6">
+        <v>26.693000000000001</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H27" s="11">
+        <f>ROUND(H25*2%, 2)</f>
+        <v>179</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K27" s="10">
+        <f>ROUND(H27*E27, 2)</f>
+        <v>4778.05</v>
+      </c>
+    </row>
     <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="31" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B31" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E31" s="6">
-        <f>ROUND(+K25/E25,2)</f>
-        <v>8949.7999999999993</v>
-      </c>
       <c r="F31" s="1" t="s">
         <v>13</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="K31" s="8">
+        <f>SUM(K25:K27)</f>
+        <v>243675.06</v>
       </c>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.2">
@@ -1146,8 +1183,8 @@
         <v>17</v>
       </c>
       <c r="K35" s="8">
-        <f>SUM(K25,K33)</f>
-        <v>62723.210000000021</v>
+        <f>SUM(K31,K33)</f>
+        <v>67501.260000000009</v>
       </c>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.2">
@@ -1162,7 +1199,7 @@
       </c>
       <c r="K36" s="10">
         <f>+K35*I36/100</f>
-        <v>3449.7765500000014</v>
+        <v>3712.5693000000006</v>
       </c>
     </row>
     <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1172,7 +1209,7 @@
       </c>
       <c r="K38" s="9">
         <f>SUM(K35:K36)</f>
-        <v>66172.986550000016</v>
+        <v>71213.829300000012</v>
       </c>
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.2">
@@ -1197,16 +1234,16 @@
     </row>
     <row r="50" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B50" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="51" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B51" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H51" s="8">
         <f>+K38</f>
-        <v>66172.986550000016</v>
+        <v>71213.829300000012</v>
       </c>
     </row>
   </sheetData>
@@ -1215,7 +1252,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0742F98C-BE43-4AE4-875B-76E1058B8CF2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4D47068-C733-464D-BF16-6D7C095707CF}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1235,22 +1272,22 @@
   <sheetData>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F8" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F9" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F10" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -1273,7 +1310,7 @@
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="2:11" ht="15" x14ac:dyDescent="0.25">
@@ -1311,15 +1348,15 @@
     </row>
     <row r="26" spans="2:11" ht="15" x14ac:dyDescent="0.25">
       <c r="B26" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C26" s="11">
+        <v>47</v>
+      </c>
+      <c r="C26" s="12">
         <v>74</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="13">
         <v>2.9870000000000001</v>
       </c>
       <c r="F26" s="3" t="s">
@@ -1440,12 +1477,12 @@
     </row>
     <row r="50" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B50" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B51" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H51" s="8">
         <f>+K38</f>
@@ -1458,7 +1495,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C0C6CB2-E0EA-43A6-B9F9-077E52785AB7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FE5D125-EDE5-45C2-A211-B2294FD6EB49}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1478,22 +1515,22 @@
   <sheetData>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F8" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F9" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F10" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -1516,7 +1553,7 @@
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="2:11" ht="15" x14ac:dyDescent="0.25">
@@ -1554,15 +1591,15 @@
     </row>
     <row r="26" spans="2:11" ht="15" x14ac:dyDescent="0.25">
       <c r="B26" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C26" s="11">
+        <v>47</v>
+      </c>
+      <c r="C26" s="12">
         <v>5</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="13">
         <v>0.20799999999999999</v>
       </c>
       <c r="F26" s="3" t="s">
@@ -1683,12 +1720,12 @@
     </row>
     <row r="50" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B50" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="51" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B51" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H51" s="8">
         <f>+K38</f>

</xml_diff>

<commit_message>
Montant des rappels avec prime.
</commit_message>
<xml_diff>
--- a/Documents/Rappels/Rappels_2402.xlsx
+++ b/Documents/Rappels/Rappels_2402.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dossier Dev\Informatique\Gestcom\Documents\Rappels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5EA33D97-C42D-4365-9E95-488695ED1F3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E2ECCE6-6F36-491F-88A7-E87043FDCF70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2325" yWindow="2235" windowWidth="21600" windowHeight="11295" firstSheet="3" activeTab="5" xr2:uid="{D8AA5B2E-01EC-4C7C-8379-53BCEF521989}"/>
+    <workbookView xWindow="2460" yWindow="1695" windowWidth="21600" windowHeight="11295" firstSheet="3" activeTab="5" xr2:uid="{53BE23F8-EDA5-44E1-91B3-628CDB5F539D}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="56">
   <si>
     <t xml:space="preserve">M PONCET FREDERIC        </t>
   </si>
@@ -58,7 +58,7 @@
     <t xml:space="preserve">      TB/PB</t>
   </si>
   <si>
-    <t>Le 17 juillet 2024</t>
+    <t>Le 19 juillet 2024</t>
   </si>
   <si>
     <t>Monsieur le Président</t>
@@ -300,11 +300,11 @@
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -645,7 +645,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE24BD8-54CD-41F6-8DAB-4C8E81FDCD62}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C352FEAB-C2FD-4C26-B9E1-A92AA298D873}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -654,7 +654,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C598DBA3-A243-4CD2-A8BF-CEB75FEC3D0E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D65A5729-2FBE-44A2-8E89-E1B2BF26453A}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -765,7 +765,7 @@
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K33" s="10">
+      <c r="K33" s="11">
         <v>-46120.800000000003</v>
       </c>
     </row>
@@ -789,7 +789,7 @@
       <c r="J36" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K36" s="10">
+      <c r="K36" s="11">
         <f>+K35*I36/100</f>
         <v>1449.0542</v>
       </c>
@@ -844,7 +844,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F71F4056-B0CA-47D0-9DBC-DDC50849DC3B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA348050-9E85-4AA3-9D94-72F50EAFC8E5}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -955,7 +955,7 @@
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K33" s="10">
+      <c r="K33" s="11">
         <v>-88294.8</v>
       </c>
     </row>
@@ -979,7 +979,7 @@
       <c r="J36" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K36" s="10">
+      <c r="K36" s="11">
         <f>+K35*I36/100</f>
         <v>1372.6454500000002</v>
       </c>
@@ -1034,7 +1034,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{401BF789-4F56-4F39-A2AC-AAB156D504D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E905546-719B-47E8-9ABC-8CC7B3BBB03F}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1141,23 +1141,33 @@
       <c r="G27" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H27" s="11">
+      <c r="H27" s="7">
         <f>ROUND(H25*2%, 2)</f>
         <v>179</v>
       </c>
+      <c r="I27" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="J27" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K27" s="10">
+      <c r="K27" s="8">
         <f>ROUND(H27*E27, 2)</f>
         <v>4778.05</v>
       </c>
+    </row>
+    <row r="28" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K28" s="10"/>
     </row>
     <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="31" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B31" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="E31" s="6">
+        <f>ROUND(K31/E25,2)</f>
+        <v>9128.7999999999993</v>
+      </c>
       <c r="F31" s="1" t="s">
         <v>13</v>
       </c>
@@ -1173,7 +1183,7 @@
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K33" s="10">
+      <c r="K33" s="11">
         <v>-176173.8</v>
       </c>
     </row>
@@ -1197,7 +1207,7 @@
       <c r="J36" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K36" s="10">
+      <c r="K36" s="11">
         <f>+K35*I36/100</f>
         <v>3712.5693000000006</v>
       </c>
@@ -1252,7 +1262,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4D47068-C733-464D-BF16-6D7C095707CF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA151D4B-D707-4474-8D37-8BB3F1FE9219}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1374,7 +1384,7 @@
       <c r="J26" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K26" s="10">
+      <c r="K26" s="11">
         <f>ROUND(+E26*H26, 2)</f>
         <v>20895.86</v>
       </c>
@@ -1416,7 +1426,7 @@
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K33" s="10">
+      <c r="K33" s="11">
         <v>0</v>
       </c>
     </row>
@@ -1440,7 +1450,7 @@
       <c r="J36" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K36" s="10">
+      <c r="K36" s="11">
         <f>+K35*I36/100</f>
         <v>10269.794699999999</v>
       </c>
@@ -1495,7 +1505,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FE5D125-EDE5-45C2-A211-B2294FD6EB49}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94DE0F3E-4491-4B0C-AAB3-3362DC342DFF}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1617,7 +1627,7 @@
       <c r="J26" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K26" s="10">
+      <c r="K26" s="11">
         <f>ROUND(+E26*H26, 2)</f>
         <v>1469.64</v>
       </c>
@@ -1659,7 +1669,7 @@
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K33" s="10">
+      <c r="K33" s="11">
         <v>0</v>
       </c>
     </row>
@@ -1683,7 +1693,7 @@
       <c r="J36" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K36" s="10">
+      <c r="K36" s="11">
         <f>+K35*I36/100</f>
         <v>6968.4780000000001</v>
       </c>

</xml_diff>

<commit_message>
Modification de l'entête des fichiers excels.
</commit_message>
<xml_diff>
--- a/Documents/Rappels/Rappels_2402.xlsx
+++ b/Documents/Rappels/Rappels_2402.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dossier Dev\Informatique\Gestcom\Documents\Rappels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E2ECCE6-6F36-491F-88A7-E87043FDCF70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{25C55C8E-73DB-4067-8A75-DC486437E79B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2460" yWindow="1695" windowWidth="21600" windowHeight="11295" firstSheet="3" activeTab="5" xr2:uid="{53BE23F8-EDA5-44E1-91B3-628CDB5F539D}"/>
+    <workbookView xWindow="-24420" yWindow="2385" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="6" xr2:uid="{0E9AC34A-668C-4B9C-B5A4-3A452932D186}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
     <sheet name="SCAF GRANGE DE VAIVRE    " sheetId="2" r:id="rId2"/>
     <sheet name="SCAF BRESSE JURASSIENNE  " sheetId="3" r:id="rId3"/>
-    <sheet name="COOP MONTS DE JOUX" sheetId="4" r:id="rId4"/>
+    <sheet name="ANDELOT" sheetId="4" r:id="rId4"/>
     <sheet name="SCAF LONGEVELLE-RUSSEY   " sheetId="5" r:id="rId5"/>
-    <sheet name="SCAF LAVANS VUILLAFANS   " sheetId="6" r:id="rId6"/>
+    <sheet name="GD COMBE CHATELEU        " sheetId="6" r:id="rId6"/>
+    <sheet name="SCAF LAVANS VUILLAFANS   " sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,12 +42,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="56">
-  <si>
-    <t xml:space="preserve">M PONCET FREDERIC        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCAF GRANGE DE VAIVRE    </t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="59">
+  <si>
+    <t>SCAF DE LA FRUITIERE DU VAL DE LOUE</t>
+  </si>
+  <si>
+    <t>Mr Frédéric PONCET</t>
   </si>
   <si>
     <t xml:space="preserve">                         </t>
@@ -58,7 +59,7 @@
     <t xml:space="preserve">      TB/PB</t>
   </si>
   <si>
-    <t>Le 19 juillet 2024</t>
+    <t>Le 23 juillet 2024</t>
   </si>
   <si>
     <t>Monsieur le Président</t>
@@ -121,40 +122,40 @@
     <t>Service Comptabilité</t>
   </si>
   <si>
-    <t>PS : Nous virons ce jour, sur votre compte N° 12506 39029 50546581010 50</t>
+    <t>PS : Nous virons ce jour, sur votre compte N° 12506 39029 50546581010 11</t>
   </si>
   <si>
     <t>CAFC SALINS LES BAINS   , la somme de</t>
   </si>
   <si>
-    <t xml:space="preserve">M BUATOIS ANTHONY        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCAF BRESSE JURASSIENNE  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 PLACE DE LA MAIRIE     </t>
+    <t>SCAF BRESSE JURASSIENNE</t>
+  </si>
+  <si>
+    <t>Mr Benoit COTE</t>
+  </si>
+  <si>
+    <t>3 Pace de la Mairie</t>
   </si>
   <si>
     <t xml:space="preserve">39140  DESNES                  </t>
   </si>
   <si>
-    <t>PS : Nous virons ce jour, sur votre compte N° 12506 39023 40357496000 40</t>
+    <t>PS : Nous virons ce jour, sur votre compte N° 12506 39023 40357496000 54</t>
   </si>
   <si>
     <t>CAFC POLIGNY            , la somme de</t>
   </si>
   <si>
+    <t>COOPERATIVE DES MONTS DE JOUX</t>
+  </si>
+  <si>
     <t>ATELIER ANDELOT</t>
   </si>
   <si>
-    <t>COOP MONTS DE JOUX</t>
-  </si>
-  <si>
-    <t>36, Rue Laurent TROUTET</t>
-  </si>
-  <si>
-    <t>25560 BANNANS</t>
+    <t>36 Rue Laurent Troutet</t>
+  </si>
+  <si>
+    <t>25560  BANANS</t>
   </si>
   <si>
     <t>Prime qualité:</t>
@@ -163,22 +164,22 @@
     <t>Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PS : Nous virons ce jour, sur votre compte N° 0 0  </t>
-  </si>
-  <si>
-    <t>, la somme de</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mr DEVAUX JOHANN         </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCAF LONGEVELLE/RUSSEY   </t>
+    <t xml:space="preserve">PS : Nous virons ce jour, sur votre compte N° 0 0               </t>
+  </si>
+  <si>
+    <t xml:space="preserve">                        , la somme de</t>
+  </si>
+  <si>
+    <t>SCAF DE LONGEVELLE</t>
+  </si>
+  <si>
+    <t>Mr Johann DEVAUX</t>
   </si>
   <si>
     <t xml:space="preserve">2, rue du Conot          </t>
   </si>
   <si>
-    <t>25380 CHARMOILLE</t>
+    <t xml:space="preserve">25380  CHARMOILLE              </t>
   </si>
   <si>
     <t>lot de fabrication JANVIER 2024 s'établit comme suit :</t>
@@ -187,25 +188,34 @@
     <t>B</t>
   </si>
   <si>
-    <t>PS : Nous virons ce jour, sur votre compte N° 12506 20017 11707951010 11</t>
+    <t>PS : Nous virons ce jour, sur votre compte N° 12506 20017 11707951010 37</t>
   </si>
   <si>
     <t>CAFC SANCEY LE GRAND    , la somme de</t>
   </si>
   <si>
-    <t xml:space="preserve">MR JOANY LEPINE          </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCAF LAVANS VUILLAFANS   </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6, Chemin des Clos Ronds </t>
+    <t>Atelier Gd Combe Chateleu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25560 BANNANS                  </t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>SCAF DE LAVANS VUILLAFANS</t>
+  </si>
+  <si>
+    <t>Mr Joany LEPINE</t>
+  </si>
+  <si>
+    <t>6 Chemin des Clos Ronds</t>
   </si>
   <si>
     <t xml:space="preserve">25380  LAVANS VUILLAFANS       </t>
   </si>
   <si>
-    <t>PS : Nous virons ce jour, sur votre compte N° 10807 6 22321737995 22</t>
+    <t>PS : Nous virons ce jour, sur votre compte N° 10807 6 22321737995 58</t>
   </si>
   <si>
     <t>BNP ORNANS              , la somme de</t>
@@ -215,10 +225,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#\ ##0.000"/>
     <numFmt numFmtId="165" formatCode="#\ ##0.00"/>
     <numFmt numFmtId="166" formatCode="#\ ##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="167" formatCode="#\ ##0.00&quot;€&quot;"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -271,7 +282,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -310,6 +321,15 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -645,7 +665,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C352FEAB-C2FD-4C26-B9E1-A92AA298D873}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{510D3903-BFFB-49B3-842E-19B5CB5457C7}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -654,7 +674,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D65A5729-2FBE-44A2-8E89-E1B2BF26453A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05360CD9-8243-44BB-A6AE-D162C024CCF1}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -844,7 +864,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA348050-9E85-4AA3-9D94-72F50EAFC8E5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A9852C5-B9A5-4B4A-BB21-9897D6EFC76E}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1034,7 +1054,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E905546-719B-47E8-9ABC-8CC7B3BBB03F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA7283FD-F39E-4DCF-A84F-E4F819B815D8}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1262,7 +1282,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA151D4B-D707-4474-8D37-8BB3F1FE9219}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14544654-7C2A-4DE3-A691-FE9F910BEAC8}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1427,7 +1447,7 @@
         <v>16</v>
       </c>
       <c r="K33" s="11">
-        <v>0</v>
+        <v>-152651.4</v>
       </c>
     </row>
     <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1437,7 +1457,7 @@
       </c>
       <c r="K35" s="8">
         <f>SUM(K27,K33)</f>
-        <v>186723.53999999998</v>
+        <v>34072.139999999985</v>
       </c>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.2">
@@ -1452,7 +1472,7 @@
       </c>
       <c r="K36" s="11">
         <f>+K35*I36/100</f>
-        <v>10269.794699999999</v>
+        <v>1873.967699999999</v>
       </c>
     </row>
     <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1462,7 +1482,7 @@
       </c>
       <c r="K38" s="9">
         <f>SUM(K35:K36)</f>
-        <v>196993.33469999998</v>
+        <v>35946.107699999986</v>
       </c>
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.2">
@@ -1496,7 +1516,7 @@
       </c>
       <c r="H51" s="8">
         <f>+K38</f>
-        <v>196993.33469999998</v>
+        <v>35946.107699999986</v>
       </c>
     </row>
   </sheetData>
@@ -1505,7 +1525,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94DE0F3E-4491-4B0C-AAB3-3362DC342DFF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3028C8E-E314-4D2F-996E-47E62289CF3C}">
   <dimension ref="A8:K51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1525,22 +1545,333 @@
   <sheetData>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F8" s="1" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F9" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F10" s="1" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B20" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B22" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B23" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+      <c r="B25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="4">
+        <v>220</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" s="5">
+        <v>8.4420000000000002</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H25" s="7">
+        <v>8949.7999999999993</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K25" s="8">
+        <f>ROUND(+E25*H25, 2)</f>
+        <v>75554.210000000006</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+      <c r="B26" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" s="4">
+        <v>10</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E26" s="5">
+        <v>0.38400000000000001</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H26" s="7">
+        <v>8000</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K26" s="8">
+        <f>ROUND(+E26*H26, 2)</f>
+        <v>3072</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+      <c r="B27" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="12">
+        <v>10</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E27" s="13">
+        <v>0.38400000000000001</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H27" s="7">
+        <v>7000</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K27" s="11">
+        <f>ROUND(+E27*H27, 2)</f>
+        <v>2688</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+      <c r="C28" s="4">
+        <f>SUM(C25:C27)</f>
+        <v>240</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E28" s="5">
+        <f>SUM(E25:E27)</f>
+        <v>9.2100000000000009</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K28" s="14">
+        <f>SUM(K25:K27)</f>
+        <v>81314.210000000006</v>
+      </c>
+    </row>
+    <row r="29" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B29" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E29" s="6">
+        <v>9.2100000000000009</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H29" s="7">
+        <f>ROUND((H25+H26+H27)*2%, 2)</f>
+        <v>479</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K29" s="16">
+        <f>ROUND(H29*E29, 2)</f>
+        <v>4411.59</v>
+      </c>
+    </row>
+    <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B31" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E31" s="6">
+        <f>ROUND(K28/E28,2)</f>
+        <v>8828.9</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="K31" s="15">
+        <f>SUM(K28:K29)</f>
+        <v>85725.8</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="D33" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K33" s="11">
+        <v>-60786</v>
+      </c>
+    </row>
+    <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="G35" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K35" s="8">
+        <f>SUM(K31:K33)</f>
+        <v>24939.800000000003</v>
+      </c>
+    </row>
+    <row r="36" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="G36" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K36" s="11">
+        <f>+K35*I36/100</f>
+        <v>1371.6890000000003</v>
+      </c>
+    </row>
+    <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="38" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+      <c r="G38" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K38" s="9">
+        <f>ROUND(SUM(K35:K36), 2)</f>
+        <v>26311.49</v>
+      </c>
+    </row>
+    <row r="40" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B40" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="42" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B42" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="43" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B43" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="45" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+      <c r="H45" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="50" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B50" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="51" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B51" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H51" s="8">
+        <f>+K38</f>
+        <v>26311.49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77498423-BBB4-48B7-9678-3BC3D217B440}">
+  <dimension ref="A8:K51"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="4.28515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="3.28515625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="11.42578125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F8" s="1" t="s">
         <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F9" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F10" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F11" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -1670,7 +2001,7 @@
         <v>16</v>
       </c>
       <c r="K33" s="11">
-        <v>0</v>
+        <v>-101521.2</v>
       </c>
     </row>
     <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1680,7 +2011,7 @@
       </c>
       <c r="K35" s="8">
         <f>SUM(K27,K33)</f>
-        <v>126699.6</v>
+        <v>25178.400000000009</v>
       </c>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.2">
@@ -1695,7 +2026,7 @@
       </c>
       <c r="K36" s="11">
         <f>+K35*I36/100</f>
-        <v>6968.4780000000001</v>
+        <v>1384.8120000000004</v>
       </c>
     </row>
     <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1705,7 +2036,7 @@
       </c>
       <c r="K38" s="9">
         <f>SUM(K35:K36)</f>
-        <v>133668.07800000001</v>
+        <v>26563.21200000001</v>
       </c>
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.2">
@@ -1730,16 +2061,16 @@
     </row>
     <row r="50" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B50" s="1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="51" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B51" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H51" s="8">
         <f>+K38</f>
-        <v>133668.07800000001</v>
+        <v>26563.21200000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modification ordre datagrid et resize la mainwindow.
</commit_message>
<xml_diff>
--- a/Documents/Rappels/Rappels_2402.xlsx
+++ b/Documents/Rappels/Rappels_2402.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dossier Dev\Informatique\Gestcom\Documents\Rappels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WpfProject\Gestcom\Documents\Rappels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1C9DA667-C164-4598-82F0-1434593A53EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9B022273-D4BD-43CA-BF2A-12DEB689BE04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24225" yWindow="3315" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="6" xr2:uid="{BFB1C835-2A59-4566-B6FB-CB60003501CF}"/>
+    <workbookView xWindow="4128" yWindow="3396" windowWidth="17280" windowHeight="8964" firstSheet="5" activeTab="6" xr2:uid="{FCF188BF-FDAF-4E4C-91C3-B84424F5A6CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
     <t xml:space="preserve">      TB/PB</t>
   </si>
   <si>
-    <t>Le 26 juillet 2024</t>
+    <t>Le 30 juillet 2024</t>
   </si>
   <si>
     <t>Monsieur le Président</t>
@@ -652,54 +652,54 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECFD12E9-13DC-449F-887F-78EC8082A57D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{768A0FAB-151E-4201-8D17-A28B7B7B3834}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3547CF28-10BC-4D6D-ABC5-2B6DD0F7D82F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7671931C-1A63-41E7-8B71-96151AD4A2A9}">
   <dimension ref="A8:K51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="4.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5.140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="3.28515625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="11.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="4.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.21875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.21875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="3.33203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.77734375" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F8" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F9" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F10" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F11" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>4</v>
       </c>
@@ -707,22 +707,22 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
         <v>9</v>
       </c>
@@ -755,8 +755,8 @@
         <v>72467.240000000005</v>
       </c>
     </row>
-    <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>15</v>
       </c>
@@ -768,7 +768,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
@@ -776,8 +776,8 @@
         <v>-46120.800000000003</v>
       </c>
     </row>
-    <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G35" s="1" t="s">
         <v>17</v>
       </c>
@@ -786,7 +786,7 @@
         <v>26346.440000000002</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G36" s="1" t="s">
         <v>18</v>
       </c>
@@ -801,8 +801,8 @@
         <v>1449.0542</v>
       </c>
     </row>
-    <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G38" s="3" t="s">
         <v>21</v>
       </c>
@@ -811,32 +811,32 @@
         <v>27795.494200000001</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B42" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B43" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
       <c r="H45" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B50" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B51" s="1" t="s">
         <v>27</v>
       </c>
@@ -851,45 +851,45 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3462FFD-3DA2-4FCE-BFD1-E1AC54E3F58F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{594F005E-60CF-492C-8A42-A20E7F596DF1}">
   <dimension ref="A8:K51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="4.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5.140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="3.28515625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="11.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="4.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.21875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.21875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="3.33203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.77734375" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F8" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F9" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F10" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F11" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>4</v>
       </c>
@@ -897,22 +897,22 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
         <v>9</v>
       </c>
@@ -945,8 +945,8 @@
         <v>113251.99</v>
       </c>
     </row>
-    <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>15</v>
       </c>
@@ -958,7 +958,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
@@ -966,8 +966,8 @@
         <v>-88294.8</v>
       </c>
     </row>
-    <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G35" s="1" t="s">
         <v>17</v>
       </c>
@@ -976,7 +976,7 @@
         <v>24957.190000000002</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G36" s="1" t="s">
         <v>18</v>
       </c>
@@ -991,8 +991,8 @@
         <v>1372.6454500000002</v>
       </c>
     </row>
-    <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G38" s="3" t="s">
         <v>21</v>
       </c>
@@ -1001,32 +1001,32 @@
         <v>26329.835450000002</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B42" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B43" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
       <c r="H45" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B50" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B51" s="1" t="s">
         <v>33</v>
       </c>
@@ -1041,45 +1041,45 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DD2F995-510F-4D6C-B472-8361D049545F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{146B3E54-8912-4CFD-83BD-8B27A1177CF3}">
   <dimension ref="A8:K51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="4.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5.140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="3.28515625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="11.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="4.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.21875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.21875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="3.33203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.77734375" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F8" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F9" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F10" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F11" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>4</v>
       </c>
@@ -1087,22 +1087,22 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
         <v>9</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>238897.01</v>
       </c>
     </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
         <v>38</v>
       </c>
@@ -1163,11 +1163,11 @@
         <v>4778.05</v>
       </c>
     </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
       <c r="K28" s="10"/>
     </row>
-    <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>15</v>
       </c>
@@ -1186,7 +1186,7 @@
         <v>243675.06</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
@@ -1194,8 +1194,8 @@
         <v>-176173.8</v>
       </c>
     </row>
-    <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G35" s="1" t="s">
         <v>17</v>
       </c>
@@ -1204,7 +1204,7 @@
         <v>67501.260000000009</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G36" s="1" t="s">
         <v>18</v>
       </c>
@@ -1219,8 +1219,8 @@
         <v>3712.5693000000006</v>
       </c>
     </row>
-    <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G38" s="3" t="s">
         <v>21</v>
       </c>
@@ -1229,32 +1229,32 @@
         <v>71213.829300000012</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B42" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B43" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
       <c r="H45" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B50" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B51" s="1" t="s">
         <v>41</v>
       </c>
@@ -1269,45 +1269,45 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70993E18-C81D-4C30-A0B3-E2FB29073D2A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1BCC41A-CDDD-42B9-A90B-FF46E6592283}">
   <dimension ref="A8:K51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="4.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5.140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="3.28515625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="11.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="4.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.21875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.21875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="3.33203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.77734375" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F8" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F9" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F10" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F11" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>4</v>
       </c>
@@ -1315,22 +1315,22 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
         <v>9</v>
       </c>
@@ -1363,7 +1363,7 @@
         <v>165827.68</v>
       </c>
     </row>
-    <row r="26" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B26" s="2" t="s">
         <v>47</v>
       </c>
@@ -1396,7 +1396,7 @@
         <v>20895.86</v>
       </c>
     </row>
-    <row r="27" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C27" s="4">
         <f>SUM(C25:C26)</f>
         <v>573</v>
@@ -1416,8 +1416,8 @@
         <v>186723.53999999998</v>
       </c>
     </row>
-    <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>15</v>
       </c>
@@ -1429,7 +1429,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
@@ -1437,8 +1437,8 @@
         <v>-152651.4</v>
       </c>
     </row>
-    <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G35" s="1" t="s">
         <v>17</v>
       </c>
@@ -1447,7 +1447,7 @@
         <v>34072.139999999985</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G36" s="1" t="s">
         <v>18</v>
       </c>
@@ -1462,8 +1462,8 @@
         <v>1873.967699999999</v>
       </c>
     </row>
-    <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G38" s="3" t="s">
         <v>21</v>
       </c>
@@ -1472,32 +1472,32 @@
         <v>35946.107699999986</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B42" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B43" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
       <c r="H45" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B50" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B51" s="1" t="s">
         <v>49</v>
       </c>
@@ -1512,45 +1512,45 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1631CA3D-DA12-483C-BBED-FF7E7AFEDBE0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06B6FDCB-27DB-407B-A196-C82060BB839C}">
   <dimension ref="A8:K51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="4.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5.140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="3.28515625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="11.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="4.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.21875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.21875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="3.33203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.77734375" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F8" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F9" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F10" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F11" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>4</v>
       </c>
@@ -1558,22 +1558,22 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
         <v>9</v>
       </c>
@@ -1606,7 +1606,7 @@
         <v>82427.66</v>
       </c>
     </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
         <v>38</v>
       </c>
@@ -1634,11 +1634,11 @@
         <v>1648.59</v>
       </c>
     </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
       <c r="K28" s="10"/>
     </row>
-    <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>15</v>
       </c>
@@ -1657,7 +1657,7 @@
         <v>84076.25</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
@@ -1665,8 +1665,8 @@
         <v>-60786</v>
       </c>
     </row>
-    <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G35" s="1" t="s">
         <v>17</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>23290.25</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G36" s="1" t="s">
         <v>18</v>
       </c>
@@ -1690,8 +1690,8 @@
         <v>1280.9637499999999</v>
       </c>
     </row>
-    <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G38" s="3" t="s">
         <v>21</v>
       </c>
@@ -1700,32 +1700,32 @@
         <v>24571.213749999999</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B42" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B43" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
       <c r="H45" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B50" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B51" s="1" t="s">
         <v>41</v>
       </c>
@@ -1740,45 +1740,45 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C40DBA2C-8D9C-4F7C-B8CD-22DA69D4BB67}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73CD2605-F925-45C5-9EB7-48901F4BDFBF}">
   <dimension ref="A8:K51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="4.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5.140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="3.28515625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="11.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="4.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.21875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.21875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="3.33203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.77734375" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F8" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F9" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F10" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F11" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>4</v>
       </c>
@@ -1786,22 +1786,22 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
         <v>9</v>
       </c>
@@ -1834,7 +1834,7 @@
         <v>125229.96</v>
       </c>
     </row>
-    <row r="26" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B26" s="2" t="s">
         <v>47</v>
       </c>
@@ -1867,7 +1867,7 @@
         <v>1469.64</v>
       </c>
     </row>
-    <row r="27" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C27" s="4">
         <f>SUM(C25:C26)</f>
         <v>369</v>
@@ -1887,8 +1887,8 @@
         <v>126699.6</v>
       </c>
     </row>
-    <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>15</v>
       </c>
@@ -1900,7 +1900,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D33" s="1" t="s">
         <v>16</v>
       </c>
@@ -1908,8 +1908,8 @@
         <v>-101521.2</v>
       </c>
     </row>
-    <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G35" s="1" t="s">
         <v>17</v>
       </c>
@@ -1918,7 +1918,7 @@
         <v>25178.400000000009</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G36" s="1" t="s">
         <v>18</v>
       </c>
@@ -1933,8 +1933,8 @@
         <v>1384.8120000000004</v>
       </c>
     </row>
-    <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G38" s="3" t="s">
         <v>21</v>
       </c>
@@ -1943,32 +1943,32 @@
         <v>26563.21200000001</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B42" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B43" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
       <c r="H45" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B50" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B51" s="1" t="s">
         <v>57</v>
       </c>

</xml_diff>